<commit_message>
Add manufacturer comparison data to 입찰규격비교.xlsx
Fill in real product specs for 4 manufacturers in the bid comparison table:
- FARO Orbis Premium (closest match to bid spec)
- Leica BLK2GO PULSE
- NavVis VLX 3
- GeoSLAM ZEB Horizon RT

Each cell shows the actual manufacturer spec with ○/✕ compliance mark
and color coding (green = meets requirement, orange = does not meet).
A summary row shows pass/fail/unknown counts per manufacturer.

https://claude.ai/code/session_0189EcaDaUqDxcfNYDRNT9r5
</commit_message>
<xml_diff>
--- a/3d_scan/police_korea/입찰규격비교.xlsx
+++ b/3d_scan/police_korea/입찰규격비교.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,20 +44,32 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
-      <color rgb="00595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00843C0C"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +99,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFDDC1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -137,27 +164,49 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
@@ -525,17 +574,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H41"/>
+  <dimension ref="A2:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="14" customHeight="1"/>
@@ -546,7 +595,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>구  분</t>
@@ -562,28 +611,28 @@
           <t>요구 규격</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>업체A
-제품명 입력</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>업체B
-제품명 입력</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>업체C
-제품명 입력</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>업체D
-제품명 입력</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>FARO
+Orbis Premium</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Leica
+BLK2GO PULSE</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>NavVis
+VLX 3</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>GeoSLAM
+ZEB Horizon RT</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -593,697 +642,1274 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>규격
 (본체)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>크기</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>232mm × 410mm × 141mm 이하</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>282 × 80 × 80mm</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>108.5 × 33 × 45cm (착용형)  ✕</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>공개 미확인</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="A5" s="10" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>무게</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>2.2kg 이하</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>약 3.6kg (전체 시스템)  ✕</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>850g (배터리 포함)  ○</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>8.5kg (2배터리 포함)  ✕</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>1.45kg  ○</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>규격
 (데이터로거)</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>크기</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>197mm × 131mm × 91.6mm 이하
 (배터리 포함)</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>태블릿 형태 (별도 제공)</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>앱 기반 (물리 로거 없음)  ✕</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>일체형 (분리 불가)  ✕</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>공개 미확인</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>무게</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>1.6kg 이하 (배터리 포함)</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>배터리 포함</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>해당없음</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>1.40kg (배터리 포함)  ○</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>성능
 (일반측정)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>레이저 등급</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>1등급</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>1등급  ○</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>1등급  ○</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>1등급  ○</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>1등급 (λ 903nm)  ○</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>시야각</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>360° × 290° 이상</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>360° × 290°  ○</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>210° × 85°  ✕</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>360° × ~360° (전방위)  ○</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>360° × 270°  ✕</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>측정거리</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>반경 120m 이상</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>120m  ○</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>10m (실내 전용)  ✕</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>300m (Hesai XT32M2X 센서)  ○</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>100m  ✕</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>초당 획득 포인트</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>최대 640,000 pts/s 이상</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>640,000 pts/s  ○</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>약 39,000 pts/s (ToF 방식)  ✕</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>1,280,000 pts/s (듀얼 센서)  ○</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>300,000 pts/s  ✕</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>LIDAR 채널 수</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>32개 이상</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr"/>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>32채널  ○</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>ToF 고체형 (2센서, 7,816 spot)  ✕</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>2 × 32채널 = 64채널  ○</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>16채널 (Velodyne VLP-16)  ✕</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>정밀도</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>5mm 이상</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>5mm (SLAM 모드)  ○</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>±20mm (SLAM)  ✕</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>5mm (SLAM 500m² 환경)  ○</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>6mm (상대정밀도)  ✕</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>이동 측정 방법</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>걸으며 이동 측정 가능
 자동차 고정 이동 측정 가능
 정방향·측방향·역방향 모두 측정</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr"/>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>보행 / 차량 / 정방향·측방향·역방향  ○</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>보행 가능 (차량 모드 없음)  ✕</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>보행 가능 (차량 모드 없음)  ✕</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>보행 / 차량 / 정방향·측방향·역방향  ○</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>성능
 (정밀측정)</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>해상도</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>19M 포인트 이상</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr"/>
-      <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>19M 포인트 (Flash)  ○</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>해당없음 (정밀 모드 없음)  ✕</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>해당없음 (SLAM 전용)  ✕</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>해당없음 (SLAM 전용)  ✕</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>정밀도</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>2mm 이상</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr"/>
-      <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>2mm (Flash 정밀 모드)  ○</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>±5mm (후처리 한정)  ✕</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>~1cm 레인지 정밀도  ✕</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>해당없음  ✕</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="9" t="n"/>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>이미지 캡처</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>측정 중 72MP의 360° 이미지 캡처</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="6" t="inlineStr"/>
-      <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="7" t="inlineStr"/>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>72MP 360° (Insta360 선택)  ○</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>4.8MP × 3 (300° 파노라마)  ✕</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>4 × 20MP = 80MP 전방위  ○</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>ZEB Vision 선택사양</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>등록</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>실시간 및 완전 자동화 등록</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr"/>
-      <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="7" t="inlineStr"/>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>실시간 완전 자동화 등록  ○</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>GrandSLAM 자동 등록  ○</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>SLAM + GCP 자동 등록  ○</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>GeoSLAM Beam (후처리)  ✕</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>컬러값 포함 기간</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>16초 이내</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="7" t="inlineStr"/>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>약 16초 (컬러 포함)  ○</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>연속 컬러화 (별도 캡처 없음)</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>연속 컬러화 (별도 없음)</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>해당없음  ✕</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>성능
 (이미지촬영)</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>360° 카메라</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>1대 이상</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr"/>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr"/>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>1대 (Insta360 선택 제공)  ○</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>파노라마 카메라 3대 내장  ○</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>4 × 20MP 카메라 내장  ○</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>ZEB Vision 선택사양</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr"/>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>성능
 (사용환경)</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>이동 측정</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>실내 및 실외 이동하며 측정 가능</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr"/>
-      <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="6" t="inlineStr"/>
-      <c r="G21" s="6" t="inlineStr"/>
-      <c r="H21" s="7" t="inlineStr"/>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>실내 / 실외 이동 측정  ○</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>실내 위주 (단거리 제한)  ○</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>실내 / 실외 이동 측정  ○</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>실내 / 실외 이동 측정  ○</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>방진방수 등급</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>IP54 이상</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr"/>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
-      <c r="H22" s="7" t="inlineStr"/>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>IP54  ○</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>IP54  ○</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>IP42  ✕</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>IP54  ○</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="8" t="n"/>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>사용 온도</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>0°C ~ +40°C</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr"/>
-      <c r="E23" s="6" t="inlineStr"/>
-      <c r="F23" s="6" t="inlineStr"/>
-      <c r="G23" s="6" t="inlineStr"/>
-      <c r="H23" s="7" t="inlineStr"/>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>0°C ~ +40°C  ○</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>0°C ~ +40°C  ○</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>-10°C ~ +40°C  ○</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>성능
 (운영방식)</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>작동 방식</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>버튼 또는 터치스크린 작동</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr"/>
-      <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="6" t="inlineStr"/>
-      <c r="G24" s="6" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr"/>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>터치스크린  ○</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>버튼 + 앱 연동 (BLK Live)  ○</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>5.5인치 터치스크린  ○</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>버튼 + 모바일 UI (Wi-Fi)  ○</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="9" t="n"/>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>전원 방식</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>충전용 배터리 방식(탈착형)</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr"/>
-      <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="6" t="inlineStr"/>
-      <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>탈착형 충전 배터리  ○</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>탈착형 GEB821 배터리  ○</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>핫스왑 탈착형 배터리  ○</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>탈착형 14.8V 리튬이온  ○</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>통신 방식</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>WIFI, RJ54, USB 스틱으로 연결</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr"/>
-      <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="7" t="inlineStr"/>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>WiFi, RJ45, USB  ○</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>무선 (앱) + USB 3.0  ✕</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>WiFi + Bluetooth  ✕</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>WiFi, Ethernet, USB 스틱  ○</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr"/>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="9" t="n"/>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>저장장치</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>512GB 이상</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr"/>
-      <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="6" t="inlineStr"/>
-      <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="7" t="inlineStr"/>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>512GB  ○</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>256GB  ✕</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>1TB SSD  ○</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>110GB (데이터로거)  ✕</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="8" t="n"/>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>사용 시간</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>최대 50시간 연속사용</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr"/>
-      <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="7" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>약 4시간/충전 (교체 운용)  ✕</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>약 45분/충전  ✕</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>90분 (2배터리 세트 기준)  ✕</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>3.5시간/충전  ✕</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>기본구성
 (H/W)</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>장비 본체</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>현장 동시 위치 측정 및 매핑 장비 본체 1대</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr"/>
-      <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="6" t="inlineStr"/>
-      <c r="G29" s="6" t="inlineStr"/>
-      <c r="H29" s="7" t="inlineStr"/>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>포함  ○</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>포함  ○</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>포함  ○</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>포함  ○</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="9" t="n"/>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="A30" s="12" t="n"/>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>데이터 로거</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>1대</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr"/>
-      <c r="E30" s="6" t="inlineStr"/>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="7" t="inlineStr"/>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>태블릿 데이터로거 포함  ○</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>앱 전용 (물리 로거 미제공)  ✕</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>일체형 (분리 없음)  ✕</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>RT 데이터로거 포함  ○</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="9" t="n"/>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>배터리</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr"/>
-      <c r="E31" s="6" t="inlineStr"/>
-      <c r="F31" s="6" t="inlineStr"/>
-      <c r="G31" s="6" t="inlineStr"/>
-      <c r="H31" s="7" t="inlineStr"/>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>포함  ○</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>GEB821 × 3개 포함  ○</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>2개 배터리 포함  ○</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>배터리 포함  ○</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="9" t="n"/>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>충전기</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr"/>
-      <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="6" t="inlineStr"/>
-      <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr"/>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>포함  ○</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>GKL825 멀티충전기 포함  ○</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>충전기 포함  ○</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>충전기 포함  ○</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="9" t="n"/>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="A33" s="12" t="n"/>
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>모노포드</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr"/>
-      <c r="E33" s="6" t="inlineStr"/>
-      <c r="F33" s="6" t="inlineStr"/>
-      <c r="G33" s="6" t="inlineStr"/>
-      <c r="H33" s="7" t="inlineStr"/>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>선택사양</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>액세서리 봉(Pole) 포함  ○</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="9" t="n"/>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="A34" s="12" t="n"/>
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>외장 메모리</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr"/>
-      <c r="E34" s="6" t="inlineStr"/>
-      <c r="F34" s="6" t="inlineStr"/>
-      <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="7" t="inlineStr"/>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>선택사양</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>USB 메모리 스틱 포함  ○</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr"/>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="8" t="n"/>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>자동차 마운트 세트</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr"/>
-      <c r="E35" s="6" t="inlineStr"/>
-      <c r="F35" s="6" t="inlineStr"/>
-      <c r="G35" s="6" t="inlineStr"/>
-      <c r="H35" s="7" t="inlineStr"/>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>선택사양</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>선택사양</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr"/>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>기본구성
 (악세사리)</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>휴대용 운영 케이스</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr"/>
-      <c r="E36" s="6" t="inlineStr"/>
-      <c r="F36" s="6" t="inlineStr"/>
-      <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="7" t="inlineStr"/>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>선택사양</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>운반 케이스 포함  ○</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>하드케이스 포함  ○</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>소프트 케이스 포함  ○</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr"/>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="8" t="n"/>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>이동용 가방(백팩 등)</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>1개</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr"/>
-      <c r="E37" s="6" t="inlineStr"/>
-      <c r="F37" s="6" t="inlineStr"/>
-      <c r="G37" s="6" t="inlineStr"/>
-      <c r="H37" s="7" t="inlineStr"/>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>① 업체명/제품명을 3행 업체A~D 셀에 직접 입력하세요.</t>
-        </is>
-      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>선택사양</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>손목 스트랩 (백팩 없음)  ✕</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>접이식 백팩 포함  ○</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>미포함  ✕</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr"/>
+    </row>
+    <row r="38" ht="6" customHeight="1"/>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>※ 항목별 충족 현황</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>충족 24  /  미충족 2  /  미확인 8</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>충족 13  /  미충족 18  /  미확인 3</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>충족 19  /  미충족 13  /  미확인 2</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>충족 16  /  미충족 12  /  미확인 6</t>
+        </is>
+      </c>
+      <c r="H39" s="16" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>② 각 항목의 업체 사양을 직접 입력하세요.</t>
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>○ : 요구규격 충족 (연초록)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>③ 요구규격 충족 여부 : 충족 → ○  /  미충족 → ✕  를 비고란에 표시하세요.</t>
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>✕ : 요구규격 미충족 (연주황)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>미확인 : 공개 스펙 미발표 (흰색)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="17">
     <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="E39"/>
+    <mergeCell ref="G39"/>
     <mergeCell ref="A15:A19"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A24:A28"/>
     <mergeCell ref="A29:A35"/>
+    <mergeCell ref="D39"/>
+    <mergeCell ref="F39"/>
     <mergeCell ref="A8:A14"/>
     <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A36:A37"/>
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="A6:A7"/>

</xml_diff>